<commit_message>
Generate comparison chart for open docks freely and open Metro first
</commit_message>
<xml_diff>
--- a/for_charts.xlsx
+++ b/for_charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Me\UofL\Data Analytics &amp; System Optimization (DASO)\MetroSafe Drone-Project\MetroSafe-UofL_Drone_Optimization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D744A2F8-3697-4716-B7D8-376F6CF0FB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3DDB03-A2C2-466E-ACBF-DC34A3C36D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="7">
   <si>
     <t>Response time (min)</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t>Open docks freely</t>
+  </si>
+  <si>
+    <t>Open MetroSafe docks first</t>
   </si>
 </sst>
 </file>
@@ -84,10 +87,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -369,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
@@ -377,18 +380,30 @@
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -404,289 +419,560 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>83.33</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>10</v>
       </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2">
+        <v>83.33</v>
+      </c>
+      <c r="I3" s="2">
+        <v>10</v>
+      </c>
+      <c r="J3" s="2">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>1.5</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>94.44</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>9</v>
       </c>
-      <c r="D4" s="3">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3">
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G4" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>94.44</v>
+      </c>
+      <c r="I4" s="2">
+        <v>9</v>
+      </c>
+      <c r="J4" s="2">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>94.44</v>
       </c>
-      <c r="C5" s="3">
-        <v>7</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="2">
+        <v>7</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>7</v>
+      </c>
+      <c r="G5" s="1">
+        <v>2</v>
+      </c>
+      <c r="H5" s="2">
+        <v>94.44</v>
+      </c>
+      <c r="I5" s="2">
+        <v>9</v>
+      </c>
+      <c r="J5" s="2">
+        <v>4</v>
+      </c>
+      <c r="K5" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>2.5</v>
       </c>
-      <c r="B6" s="3">
-        <v>100</v>
-      </c>
-      <c r="C6" s="3">
-        <v>7</v>
-      </c>
-      <c r="D6" s="3">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="2">
+        <v>100</v>
+      </c>
+      <c r="C6" s="2">
+        <v>7</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>7</v>
+      </c>
+      <c r="G6" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="H6" s="2">
+        <v>100</v>
+      </c>
+      <c r="I6" s="2">
+        <v>8</v>
+      </c>
+      <c r="J6" s="2">
+        <v>3</v>
+      </c>
+      <c r="K6" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="3">
-        <v>100</v>
-      </c>
-      <c r="C7" s="3">
-        <v>7</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="2">
+        <v>100</v>
+      </c>
+      <c r="C7" s="2">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>7</v>
+      </c>
+      <c r="G7" s="1">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2">
+        <v>100</v>
+      </c>
+      <c r="I7" s="2">
+        <v>8</v>
+      </c>
+      <c r="J7" s="2">
+        <v>4</v>
+      </c>
+      <c r="K7" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>3.5</v>
       </c>
-      <c r="B8" s="3">
-        <v>100</v>
-      </c>
-      <c r="C8" s="3">
-        <v>7</v>
-      </c>
-      <c r="D8" s="3">
-        <v>0</v>
-      </c>
-      <c r="E8" s="3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="2">
+        <v>100</v>
+      </c>
+      <c r="C8" s="2">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>7</v>
+      </c>
+      <c r="G8" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="H8" s="2">
+        <v>100</v>
+      </c>
+      <c r="I8" s="2">
+        <v>8</v>
+      </c>
+      <c r="J8" s="2">
+        <v>4</v>
+      </c>
+      <c r="K8" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>4</v>
       </c>
-      <c r="B9" s="3">
-        <v>100</v>
-      </c>
-      <c r="C9" s="3">
-        <v>7</v>
-      </c>
-      <c r="D9" s="3">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="2">
+        <v>100</v>
+      </c>
+      <c r="C9" s="2">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>7</v>
+      </c>
+      <c r="G9" s="1">
+        <v>4</v>
+      </c>
+      <c r="H9" s="2">
+        <v>100</v>
+      </c>
+      <c r="I9" s="2">
+        <v>8</v>
+      </c>
+      <c r="J9" s="2">
+        <v>4</v>
+      </c>
+      <c r="K9" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>4.5</v>
       </c>
-      <c r="B10" s="3">
-        <v>100</v>
-      </c>
-      <c r="C10" s="3">
+      <c r="B10" s="2">
+        <v>100</v>
+      </c>
+      <c r="C10" s="2">
         <v>6</v>
       </c>
-      <c r="D10" s="3">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3">
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G10" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="H10" s="2">
+        <v>100</v>
+      </c>
+      <c r="I10" s="2">
+        <v>7</v>
+      </c>
+      <c r="J10" s="2">
+        <v>3</v>
+      </c>
+      <c r="K10" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>5</v>
       </c>
-      <c r="B11" s="3">
-        <v>100</v>
-      </c>
-      <c r="C11" s="3">
+      <c r="B11" s="2">
+        <v>100</v>
+      </c>
+      <c r="C11" s="2">
         <v>5</v>
       </c>
-      <c r="D11" s="3">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3">
+      <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G11" s="1">
+        <v>5</v>
+      </c>
+      <c r="H11" s="2">
+        <v>100</v>
+      </c>
+      <c r="I11" s="2">
+        <v>5</v>
+      </c>
+      <c r="J11" s="2">
+        <v>3</v>
+      </c>
+      <c r="K11" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>5.5</v>
       </c>
-      <c r="B12" s="3">
-        <v>100</v>
-      </c>
-      <c r="C12" s="3">
-        <v>4</v>
-      </c>
-      <c r="D12" s="3">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="2">
+        <v>100</v>
+      </c>
+      <c r="C12" s="2">
+        <v>4</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>4</v>
+      </c>
+      <c r="G12" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="H12" s="2">
+        <v>100</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4</v>
+      </c>
+      <c r="J12" s="2">
+        <v>2</v>
+      </c>
+      <c r="K12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>6</v>
       </c>
-      <c r="B13" s="3">
-        <v>100</v>
-      </c>
-      <c r="C13" s="3">
-        <v>4</v>
-      </c>
-      <c r="D13" s="3">
-        <v>0</v>
-      </c>
-      <c r="E13" s="3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="2">
+        <v>100</v>
+      </c>
+      <c r="C13" s="2">
+        <v>4</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>4</v>
+      </c>
+      <c r="G13" s="1">
+        <v>6</v>
+      </c>
+      <c r="H13" s="2">
+        <v>100</v>
+      </c>
+      <c r="I13" s="2">
+        <v>4</v>
+      </c>
+      <c r="J13" s="2">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>6.5</v>
       </c>
-      <c r="B14" s="3">
-        <v>100</v>
-      </c>
-      <c r="C14" s="3">
-        <v>3</v>
-      </c>
-      <c r="D14" s="3">
-        <v>0</v>
-      </c>
-      <c r="E14" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="2">
+        <v>100</v>
+      </c>
+      <c r="C14" s="2">
+        <v>3</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>3</v>
+      </c>
+      <c r="G14" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="H14" s="2">
+        <v>100</v>
+      </c>
+      <c r="I14" s="2">
+        <v>5</v>
+      </c>
+      <c r="J14" s="2">
+        <v>3</v>
+      </c>
+      <c r="K14" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>7</v>
       </c>
-      <c r="B15" s="3">
-        <v>100</v>
-      </c>
-      <c r="C15" s="3">
-        <v>3</v>
-      </c>
-      <c r="D15" s="3">
+      <c r="B15" s="2">
+        <v>100</v>
+      </c>
+      <c r="C15" s="2">
+        <v>3</v>
+      </c>
+      <c r="D15" s="2">
         <v>1</v>
       </c>
-      <c r="E15" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E15" s="2">
+        <v>2</v>
+      </c>
+      <c r="G15" s="1">
+        <v>7</v>
+      </c>
+      <c r="H15" s="2">
+        <v>100</v>
+      </c>
+      <c r="I15" s="2">
+        <v>5</v>
+      </c>
+      <c r="J15" s="2">
+        <v>3</v>
+      </c>
+      <c r="K15" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>7.5</v>
       </c>
-      <c r="B16" s="3">
-        <v>100</v>
-      </c>
-      <c r="C16" s="3">
-        <v>3</v>
-      </c>
-      <c r="D16" s="3">
+      <c r="B16" s="2">
+        <v>100</v>
+      </c>
+      <c r="C16" s="2">
+        <v>3</v>
+      </c>
+      <c r="D16" s="2">
         <v>1</v>
       </c>
-      <c r="E16" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E16" s="2">
+        <v>2</v>
+      </c>
+      <c r="G16" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="H16" s="2">
+        <v>100</v>
+      </c>
+      <c r="I16" s="2">
+        <v>4</v>
+      </c>
+      <c r="J16" s="2">
+        <v>3</v>
+      </c>
+      <c r="K16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>8</v>
       </c>
-      <c r="B17" s="3">
-        <v>100</v>
-      </c>
-      <c r="C17" s="3">
-        <v>3</v>
-      </c>
-      <c r="D17" s="3">
-        <v>0</v>
-      </c>
-      <c r="E17" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B17" s="2">
+        <v>100</v>
+      </c>
+      <c r="C17" s="2">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>3</v>
+      </c>
+      <c r="G17" s="1">
+        <v>8</v>
+      </c>
+      <c r="H17" s="2">
+        <v>100</v>
+      </c>
+      <c r="I17" s="2">
+        <v>4</v>
+      </c>
+      <c r="J17" s="2">
+        <v>3</v>
+      </c>
+      <c r="K17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>8.5</v>
       </c>
-      <c r="B18" s="3">
-        <v>100</v>
-      </c>
-      <c r="C18" s="3">
-        <v>2</v>
-      </c>
-      <c r="D18" s="3">
-        <v>0</v>
-      </c>
-      <c r="E18" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="2">
+        <v>100</v>
+      </c>
+      <c r="C18" s="2">
+        <v>2</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0</v>
+      </c>
+      <c r="E18" s="2">
+        <v>2</v>
+      </c>
+      <c r="G18" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="H18" s="2">
+        <v>100</v>
+      </c>
+      <c r="I18" s="2">
+        <v>4</v>
+      </c>
+      <c r="J18" s="2">
+        <v>3</v>
+      </c>
+      <c r="K18" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="G19" s="1">
+        <v>9</v>
+      </c>
+      <c r="H19" s="2">
+        <v>100</v>
+      </c>
+      <c r="I19" s="2">
+        <v>2</v>
+      </c>
+      <c r="J19" s="2">
+        <v>2</v>
+      </c>
+      <c r="K19" s="2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="G1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>